<commit_message>
PAUSED (task151): stage 4 repair green, FIN-14 4.4 look-back filed, golden re-derived to $4,250,000, waiting on the re-judge
Judge round 1 (NOT_DETERMINISTIC, no filed preference among the bases) and the rule 3 audit's strength finding repaired
inside architecture 1: FIN-14 4.4 files a look-back selection criterion naming no method; the starting nines' raw
seasons now miss by 1.53 to 1.77 bins on every window; 4.3 restated, Ask B's population and attribution filed, one
rounding path, Ask A's effective date filed, the close-file index renamed; world redrawn (seed 1539). checks 276,
verify, two byte-identical builds, figures_check 87, precut 49, voice-check, container audit, leak.py REVIEW.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task151/golden/pa_bonus_accrual_2027.xlsx
+++ b/task151/golden/pa_bonus_accrual_2027.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accrual" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IL stints since 2024" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PA bonuses paid 2024-2026" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Look-back (FIN-14 4.4)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IL stints since 2024" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PA bonuses paid 2024-2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Accrual'!$5:$5</definedName>
@@ -21,13 +22,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="166" formatCode="$#,##0"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +47,7 @@
     <font>
       <i val="1"/>
     </font>
+    <font/>
   </fonts>
   <fills count="3">
     <fill>
@@ -76,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -92,6 +95,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -478,7 +483,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plate-appearance bonuses, 2027 free-agent hitters: accrual at signing $3,500,000</t>
+          <t>Plate-appearance bonuses, 2027 free-agent hitters: accrual at signing $4,250,000</t>
         </is>
       </c>
     </row>
@@ -541,271 +546,271 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jairo Calderón</t>
+          <t>Sawyer Lusk</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
         <v>46350</v>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>475</v>
+        <v>500</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>350000</v>
+        <v>320000</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.7826</v>
+        <v>0.7438</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>273923.61</v>
+        <v>238000</v>
       </c>
     </row>
     <row r="7">
       <c r="D7" t="n">
-        <v>525</v>
+        <v>575</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>350000</v>
+        <v>320000</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.7056</v>
+        <v>0.5681</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>246944.44</v>
+        <v>181777.78</v>
       </c>
     </row>
     <row r="8">
       <c r="D8" t="n">
-        <v>600</v>
+        <v>650</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>350000</v>
+        <v>320000</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>0.5083</v>
+        <v>0.2938</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>177916.67</v>
+        <v>94000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Jairo Calderón, accrual</t>
+          <t>Sawyer Lusk, accrual</t>
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>698784.72</v>
+        <v>513777.78</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>700000</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Kevin Weeks</t>
+          <t>Andres Rivas</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
         <v>46356</v>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D10" t="n">
-        <v>475</v>
+        <v>525</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>450000</v>
+        <v>750000</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>0.7632</v>
+        <v>0.6667</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>343437.5</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="11">
       <c r="D11" t="n">
-        <v>550</v>
+        <v>575</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>450000</v>
+        <v>750000</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.6104000000000001</v>
+        <v>0.5319</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>274687.5</v>
+        <v>398958.33</v>
       </c>
     </row>
     <row r="12">
       <c r="D12" t="n">
-        <v>625</v>
+        <v>650</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>450000</v>
+        <v>750000</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>0.3792</v>
+        <v>0.1493</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>170625</v>
+        <v>111979.17</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Kevin Weeks, accrual</t>
+          <t>Andres Rivas, accrual</t>
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>788750</v>
+        <v>1010937.5</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>800000</v>
+        <v>1000000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ramon Figueroa</t>
+          <t>Drew Brock</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
         <v>46359</v>
       </c>
       <c r="C14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D14" t="n">
-        <v>500</v>
+        <v>450</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>500000</v>
+        <v>330000</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>0.6986</v>
+        <v>0.791</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>349305.56</v>
+        <v>261020.83</v>
       </c>
     </row>
     <row r="15">
       <c r="D15" t="n">
-        <v>550</v>
+        <v>525</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>500000</v>
+        <v>330000</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>0.5757</v>
+        <v>0.6306</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>287847.22</v>
+        <v>208083.33</v>
       </c>
     </row>
     <row r="16">
       <c r="D16" t="n">
-        <v>625</v>
+        <v>600</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>500000</v>
+        <v>330000</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>0.3389</v>
+        <v>0.359</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>169444.44</v>
+        <v>118479.17</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Ramon Figueroa, accrual</t>
+          <t>Drew Brock, accrual</t>
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>806597.22</v>
+        <v>587583.33</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>800000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Eric Dobbs</t>
+          <t>Ángel Medina</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
         <v>46364</v>
       </c>
       <c r="C18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D18" t="n">
-        <v>525</v>
+        <v>500</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>560000</v>
+        <v>730000</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>0.6104000000000001</v>
+        <v>0.6597</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>341833.33</v>
+        <v>481597.22</v>
       </c>
     </row>
     <row r="19">
       <c r="D19" t="n">
-        <v>575</v>
+        <v>525</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>560000</v>
+        <v>730000</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>0.4549</v>
+        <v>0.5951</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>254722.22</v>
+        <v>434451.39</v>
       </c>
     </row>
     <row r="20">
       <c r="D20" t="n">
-        <v>650</v>
+        <v>575</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>560000</v>
+        <v>730000</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>0.0125</v>
+        <v>0.3868</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>7000</v>
+        <v>282368.06</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Eric Dobbs, accrual</t>
+          <t>Ángel Medina, accrual</t>
         </is>
       </c>
       <c r="G21" s="5" t="n">
-        <v>603555.5600000001</v>
+        <v>1198416.67</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>600000</v>
+        <v>1200000</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dylan Harlow</t>
+          <t>Mike Meeks</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
@@ -815,57 +820,57 @@
         <v>9</v>
       </c>
       <c r="D22" t="n">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>360000</v>
+        <v>720000</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>0.7181</v>
+        <v>0.6306</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>258500</v>
+        <v>454000</v>
       </c>
     </row>
     <row r="23">
       <c r="D23" t="n">
-        <v>500</v>
+        <v>550</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>360000</v>
+        <v>720000</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>0.5965</v>
+        <v>0.4437</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>214750</v>
+        <v>319500</v>
       </c>
     </row>
     <row r="24">
       <c r="D24" t="n">
-        <v>575</v>
+        <v>600</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>360000</v>
+        <v>720000</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>0.3472</v>
+        <v>0.191</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>125000</v>
+        <v>137500</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Dylan Harlow, accrual</t>
+          <t>Mike Meeks, accrual</t>
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>598250</v>
+        <v>911000</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>600000</v>
+        <v>900000</v>
       </c>
     </row>
     <row r="26">
@@ -875,10 +880,10 @@
         </is>
       </c>
       <c r="G26" s="5" t="n">
-        <v>3495937.5</v>
+        <v>4221715.28</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>3500000</v>
+        <v>4250000</v>
       </c>
     </row>
     <row r="28">
@@ -947,31 +952,31 @@
         </is>
       </c>
       <c r="B30" s="10" t="n">
-        <v>4.727</v>
+        <v>4.716</v>
       </c>
       <c r="C30" s="10" t="n">
-        <v>4.611</v>
+        <v>4.596</v>
       </c>
       <c r="D30" s="10" t="n">
-        <v>4.489</v>
+        <v>4.481</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>4.378</v>
+        <v>4.366</v>
       </c>
       <c r="F30" s="10" t="n">
-        <v>4.258</v>
+        <v>4.247</v>
       </c>
       <c r="G30" s="10" t="n">
-        <v>4.152</v>
+        <v>4.139</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>4.049</v>
+        <v>4.038</v>
       </c>
       <c r="I30" s="10" t="n">
-        <v>3.944</v>
+        <v>3.936</v>
       </c>
       <c r="J30" s="10" t="n">
-        <v>3.838</v>
+        <v>3.828</v>
       </c>
     </row>
   </sheetData>
@@ -981,6 +986,298 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="66" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>FIN-14 4.4 look-back: 748 hitter-seasons, 2023 to 2026; the basis with the lowest score is used</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Each basis applied to each season with what was published before it began, to every hitter in a starting lineup of that season's January 31 depth charts with 100 plate appearances in each of the two seasons before; score: the average squared difference between the probability of 450, 500, 550, 600 and 650 plate appearances and the outcome (1 reached, 0 not).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Above the basis used</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2027 accrual on this basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Non-catcher regulars' seasons of starts at the player's 2027 slot (used)</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>0.173</v>
+      </c>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="n">
+        <v>4250000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>The same, the last three seasons only</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>0.173</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>4250000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>The same, each season's plate appearances rescaled to the slot</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>0.1732</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>4250000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Vendor's projection with a normal band from its misses</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>0.2254</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.3025</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>6250000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Vendor's projection plus each of its past misses</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>0.2206</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>0.2748</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>7250000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>The player's own last three seasons</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>0.2698</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>0.5595</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>7750000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Every lineup regular's plate appearances, catchers in, any slot</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="n">
+        <v>0.2182</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>0.2609</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>4500000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Non-catcher regulars' plate appearances, any slot</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>0.1845</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>0.0665</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>5250000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Every lineup regular's starts at the player's slot, catchers in</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>0.194</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>0.1211</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>3750000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Opening-day starters' seasons at the player's slot</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>0.1766</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>0.0207</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>4000000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Regulars who started their club's first game, at the slot</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>0.1751</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>4750000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Hitters with 400 or more plate appearances, at the slot</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>0.1792</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>0.036</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>4500000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>The regulars' seasons moved 10 per cent toward the player's record</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="n">
+        <v>0.1758</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>0.0161</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>4750000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Regression on the vendor's projection, slot and catching</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="n">
+        <v>0.1749</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>0.0107</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>4250000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>The bases that tie the one used (the last three seasons; plate appearances rescaled) give the same accrual. Accruals to the nearest $250,000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sources: hvbd_winter_depth_charts_2021_2026.xlsx; hvbd_hitter_projections_2022_2027.csv; the batting lines 2021 to 2026.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1002,7 +1299,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>Injured-list stints of the five since Opening Day 2024: nine stints, 235 regular-season days</t>
+          <t>Injured-list stints of the five since Opening Day 2024: nine stints, 233 regular-season days</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1348,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jairo Calderón</t>
+          <t>Sawyer Lusk</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1076,16 +1373,16 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>45482</v>
+        <v>45484</v>
       </c>
       <c r="H4" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Eric Dobbs</t>
+          <t>Ángel Medina</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1099,10 +1396,10 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
+        <v>45432</v>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>45431</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>45430</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1113,13 +1410,13 @@
         <v>45441</v>
       </c>
       <c r="H5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Eric Dobbs</t>
+          <t>Ángel Medina</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1153,7 +1450,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Dylan Harlow</t>
+          <t>Mike Meeks</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1178,16 +1475,16 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>45522</v>
+        <v>45521</v>
       </c>
       <c r="H7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ramon Figueroa</t>
+          <t>Drew Brock</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1201,10 +1498,10 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>45521</v>
+        <v>45520</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>45519</v>
+        <v>45518</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1212,7 +1509,7 @@
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>45532</v>
+        <v>45531</v>
       </c>
       <c r="H8" t="n">
         <v>13</v>
@@ -1221,7 +1518,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dylan Harlow</t>
+          <t>Mike Meeks</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1246,16 +1543,16 @@
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>45758</v>
+        <v>45756</v>
       </c>
       <c r="H9" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ramon Figueroa</t>
+          <t>Drew Brock</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1289,7 +1586,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Kevin Weeks</t>
+          <t>Andres Rivas</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1323,7 +1620,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jairo Calderón</t>
+          <t>Sawyer Lusk</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1373,7 +1670,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1417,11 +1714,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Carson Bickford</t>
+          <t>Edwin Cedeno</t>
         </is>
       </c>
       <c r="C4" s="5" t="n">
-        <v>420000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="5">
@@ -1430,11 +1727,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Andrés Acevedo</t>
+          <t>Jonathan Vasquez</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>300000</v>
+        <v>125000</v>
       </c>
     </row>
     <row r="6">
@@ -1447,7 +1744,7 @@
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>720000</v>
+        <v>325000</v>
       </c>
     </row>
     <row r="8">
@@ -1456,11 +1753,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Zach Strickland</t>
+          <t>Jonathan Vasquez</t>
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>225000</v>
+        <v>375000</v>
       </c>
     </row>
     <row r="9">
@@ -1469,37 +1766,37 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Shota Nakagawa</t>
+          <t>Gregorio Candelario</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>100000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
         <v>2025</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Juan Nunez</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>225000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Total 2025</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n">
-        <v>325000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Elijah Mosley</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>187500</v>
+      <c r="C11" s="9" t="n">
+        <v>900000</v>
       </c>
     </row>
     <row r="13">
@@ -1508,11 +1805,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Shota Nakagawa</t>
+          <t>Jacob Briggs</t>
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>150000</v>
+        <v>262500</v>
       </c>
     </row>
     <row r="14">
@@ -1521,11 +1818,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Kody Bagwell</t>
+          <t>Gregorio Candelario</t>
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>87500</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="15">
@@ -1538,7 +1835,7 @@
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>425000</v>
+        <v>412500</v>
       </c>
     </row>
     <row r="17">
@@ -1574,7 +1871,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1587,37 +1884,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>As of December 11, 2026 (files pulled that afternoon). Prepared by Harry Barnes, Controller.</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
-        <is>
-          <t>Accrual under FIN-14 4.2 to 4.4: each plate-appearance bonus at its amount times the probability that the player reaches its threshold in the 2027 championship season, assessed at signing, the player taken as staying with the Club in his planned role (lineup slot in ral_depth_chart_2027.xlsx).</t>
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>Accrual under FIN-14 4.2 and 4.3: each plate-appearance bonus at its amount times the probability that the player reaches its threshold in the 2027 championship season, assessed at signing, the contract taken as standing all season with the player in his planned role (lineup slot in ral_depth_chart_2027.xlsx) and his health and playing time left in the probability. Basis chosen by the FIN-14 4.4 look-back (sheet Look-back).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Plate appearances as the term sheets define them: championship season, for the Club; postseason and rehabilitation-assignment plate appearances excluded.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>Comparison seasons: the non-catchers in the lineups of hvbd_winter_depth_charts_2021_2026.xlsx, 1,440 seasons; starts counted for every club the player started for that season, from lsf_batting_2021_2024.txt (through lsf_player_id_crosswalk.csv) and lsf_batting_2025_2026.csv.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>Rounding: each player's accrual to the nearest $100,000 and the total to the nearest $250,000, both from the unrounded line amounts.</t>
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Rounding (FIN-14 6): each player's accrual to the nearest $100,000 and the total to the nearest $250,000, both from the unrounded line amounts; the rounded player figures add to $4,200,000.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
RESHIPPED (task151): determinism, the ask's catch-up rows closed: the contract register's header files the payment schedule (one half in the October 15 run after the season, one half in the January 15 run after that, in full in the October 15 run after a contract's last season), so the season-by-run reading both portal judges took (White $60,000 and $180,000, Livingston $50,000 and $150,000) breaks a quoted sentence (SF23); the call, the stump and every graded figure frozen (freeze determinism PASS, target.zip 90a982cd); judge 2's open-basis point left open as the filed look-back; no re-judge on the author's instruction
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/task151/golden/pa_bonus_accrual_2027.xlsx
+++ b/task151/golden/pa_bonus_accrual_2027.xlsx
@@ -1329,12 +1329,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Season-end payment</t>
+          <t>Season-end payment for the season</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>January payment</t>
+          <t>January half for the season</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1892,7 +1892,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>The pitchers' bonuses are paid half in the season-end run (October 15) and half on the following January 15; after the last season of a contract the season-end run pays the whole season. Before the January 2026 HRIS cutover the legacy payroll put the season-end payments on E45 OTHER BONUS and the January halves on E40 PERF BONUS; from January 2026 both are BPA.</t>
+          <t>Payment terms per the contract register's note: one half in the October 15 run after the season and one half in the January 15 run after that, the whole in the October 15 run after a contract's last season. Before the January 2026 HRIS cutover the legacy payroll put the season-end payments on E45 OTHER BONUS and the January halves on E40 PERF BONUS; from January 2026 both are BPA. The January 2024 run paid no half to White and the January 2025 run none to Livingston: each half was paid in his next October line, which exceeds the January half after it by that half, and is shown here in the season it was payable for (White 2023, Livingston 2024).</t>
         </is>
       </c>
     </row>

</xml_diff>